<commit_message>
Clean up duplicate file structure
Removed old searches/prompts/ tree (duplicated in searches/joey/ and searches/For_Others/). Fixed 'Core ' folder name. Renamed Vivienne _1 file. Removed misplaced template from results/.
</commit_message>
<xml_diff>
--- a/Job_Search_Tracking.xlsx
+++ b/Job_Search_Tracking.xlsx
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -122,6 +122,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -488,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -704,27 +707,47 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Vivienne Pham</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Joey Clark</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>54</v>
+      </c>
+      <c r="E7" t="n">
+        <v>95</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Greenhouse/Lever/Ashby | CoS, Partnerships, Strat Init | Remote, MX, PA, AR</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Week_of_2026-02-16/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Edwin Jones</t>
+          <t>Vivienne Pham</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -739,6 +762,62 @@
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Edwin Jones</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Vivienne Pham</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>97</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Greenhouse / Lever / Ashby / LinkedIn</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Vivienne_Pham/Week_of_2026-02-16/</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update tracking spreadsheet and execution log
Added Feb 22 search entries for all 4 friends in Job_Search_Tracking.xlsx
and marked previous searches as completed. Added Phil's execution log.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Search_Tracking.xlsx
+++ b/Job_Search_Tracking.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -581,276 +581,388 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="3" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>22</v>
+      </c>
+      <c r="E3" t="n">
+        <v>87</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4 boards + career pages | CoS, Partnerships, BD | DC, London</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Phil_Tassi/Week_of_2026-02-16/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>2026-02-08</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>93</v>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Greenhouse/Lever/Ashby | CoS, Partnerships, BD | DC &amp; London</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-15 ✓</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>Phil_Tassi/Week_of_2026-02-02/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-15</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>40</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>93</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>Greenhouse/Lever/Ashby | CoS, Partnerships, BD | DC &amp; London</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-15 ✓</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Phil_Tassi/Week_of_2026-02-02/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>93</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>Greenhouse/Lever/Ashby/LinkedIn | CoS, Partnerships, BD | DC &amp; London</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>2026-02-22</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Phil_Tassi/Week_of_2026-02-09/</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Aaron Kimson</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>2026-02-12</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>97</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Greenhouse/Lever/Ashby/LinkedIn | L/S HF Analyst, HF PM, Dir ER, Inv Analyst | NY, SF, Chicago, Miami, Boston</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>2026-02-19 ✓</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Aaron_Kimson/Week_of_2026-02-09/</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-02-15</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>22</v>
-      </c>
-      <c r="E6" t="n">
-        <v>97</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Greenhouse/Lever/Ashby/LinkedIn | L/S HF Analyst, HF PM, Dir ER, Inv Analyst | NY, SF, CHI, BOS, CT, MIA + 16 career pages</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Aaron_Kimson/Week_of_2026-02-16/</t>
-        </is>
-      </c>
-    </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Joey Clark</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
         <v>95</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>4 boards + career pages | HF Analyst, PM, ER Dir, Inv Analyst | NY, SF, CHI, BOS, CT, MIA</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Aaron_Kimson/Week_of_2026-02-16/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>22</v>
+      </c>
+      <c r="E8" t="n">
+        <v>97</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Greenhouse/Lever/Ashby/LinkedIn | L/S HF Analyst, HF PM, Dir ER, Inv Analyst | NY, SF, CHI, BOS, CT, MIA + 16 career pages</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Aaron_Kimson/Week_of_2026-02-16/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Joey Clark</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E9" t="n">
+        <v>95</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>Greenhouse/Lever/Ashby | CoS, Partnerships, Strat Init | Remote, MX, PA, AR</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>2026-02-22</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Week_of_2026-02-16/</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Vivienne Pham</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Edwin Jones</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Vivienne Pham</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>2026-02-15</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D12" s="9" t="n">
         <v>31</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E12" s="9" t="n">
         <v>97</v>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Greenhouse / Lever / Ashby / LinkedIn</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Vivienne_Pham/Week_of_2026-02-16/ ✓</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" t="n">
+        <v>100</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>4 boards | 9 roles (3 archetypes) | NYC, DC, Remote</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>Vivienne_Pham/Week_of_2026-02-16/</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr">
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rosalind Gahamire</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>87</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Greenhouse/Lever/Ashby/LinkedIn | Brand Strategist, Creative Strategist, Marketing Manager | Lisbon, Remote-Global/EMEA</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-02-23 ✓</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Rosalind_Gahamire/Week_of_2026-02-16/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" t="inlineStr">
         <is>
           <t>2026-02-22</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Rosalind Gahamire</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-02-18</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>8</v>
-      </c>
-      <c r="E11" t="n">
+      <c r="D15" t="n">
+        <v>18</v>
+      </c>
+      <c r="E15" t="n">
         <v>87</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Greenhouse/Lever/Ashby/LinkedIn | Brand Strategist, Creative Strategist, Marketing Manager | Lisbon, Remote-Global/EMEA</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>4 boards | Brand/Creative Strategy, Marketing Mgr | Lisbon, Remote-Global</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Rosalind_Gahamire/Week_of_2026-02-16/</t>
         </is>

</xml_diff>

<commit_message>
Update job search tracking spreadsheet
</commit_message>
<xml_diff>
--- a/Job_Search_Tracking.xlsx
+++ b/Job_Search_Tracking.xlsx
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="10" min="1" max="1"/>
@@ -697,356 +697,445 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>2026-02-24</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="10" t="n">
         <v>37</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>4 boards | COS, Partnerships, BD | DC, London</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-03-02</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-02 ✓</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>Phil_Tassi/Week_of_2026-02-23/</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Aaron Kimson</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>2026-02-12</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>24</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>97</v>
-      </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>Greenhouse/Lever/Ashby/LinkedIn | L/S HF Analyst, HF PM, Dir ER, Inv Analyst | NY, SF, Chicago, Miami, Boston</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>2026-02-19 ✓</t>
-        </is>
-      </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>Aaron_Kimson/Week_of_2026-02-09/</t>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>93</v>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>4 boards | CoS, Partnerships, BD | DC, London</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-02 ✓</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Phil_Tassi/Week_of_2026-02-23/</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
       <c r="C8" s="10" t="inlineStr">
         <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>93</v>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>3 boards | COS, Partnerships, BD | DC, London</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Phil_Tassi/Week_of_2026-02-23/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="11">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Aaron Kimson</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>97</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Greenhouse/Lever/Ashby/LinkedIn | L/S HF Analyst, HF PM, Dir ER, Inv Analyst | NY, SF, Chicago, Miami, Boston</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>2026-02-19 ✓</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Aaron_Kimson/Week_of_2026-02-09/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="11">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
           <t>2026-02-22</t>
         </is>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D10" s="10" t="n">
         <v>10</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>95</v>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>4 boards + career pages | HF Analyst, PM, ER Dir, Inv Analyst | NY, SF, CHI, BOS, CT, MIA</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Aaron_Kimson/Week_of_2026-02-16/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="11">
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>2026-02-15</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>97</v>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>Greenhouse/Lever/Ashby/LinkedIn | L/S HF Analyst, HF PM, Dir ER, Inv Analyst | NY, SF, CHI, BOS, CT, MIA + 16 career pages</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Aaron_Kimson/Week_of_2026-02-16/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="11">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>Joey Clark</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>2026-02-15</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>54</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>95</v>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Greenhouse/Lever/Ashby | CoS, Partnerships, Strat Init | Remote, MX, PA, AR</t>
+          <t>4 boards + career pages | HF Analyst, PM, ER Dir, Inv Analyst | NY, SF, CHI, BOS, CT, MIA</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>2026-02-22 ✓</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>Week_of_2026-02-16/</t>
+          <t>Aaron_Kimson/Week_of_2026-02-16/</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
       <c r="C11" s="10" t="inlineStr">
         <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>97</v>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Greenhouse/Lever/Ashby/LinkedIn | L/S HF Analyst, HF PM, Dir ER, Inv Analyst | NY, SF, CHI, BOS, CT, MIA + 16 career pages</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Aaron_Kimson/Week_of_2026-02-16/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="11">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Joey Clark</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>54</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Greenhouse/Lever/Ashby | CoS, Partnerships, Strat Init | Remote, MX, PA, AR</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-22 ✓</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Week_of_2026-02-16/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="11">
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E13" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>Greenhouse, Lever, Ashby | CoS, Partnerships, Strategic Initiatives | Remote, Panama, Buenos Aires, Manila</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
         <is>
           <t>2026-03-02</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>Week_of_2026-02-23/</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="11">
-      <c r="A12" s="13" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" s="11">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Vivienne Pham</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="11">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="11">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Edwin Jones</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="13" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="11">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
+      <c r="E15" s="13" t="n"/>
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
+      <c r="H15" s="13" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="11">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Vivienne Pham</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>2026-02-15</t>
         </is>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D16" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E16" s="20" t="n">
         <v>97</v>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F16" s="20" t="inlineStr">
         <is>
           <t>Greenhouse / Lever / Ashby / LinkedIn</t>
         </is>
       </c>
-      <c r="G14" s="20" t="inlineStr">
-        <is>
-          <t>Vivienne_Pham/Week_of_2026-02-16/ ✓</t>
-        </is>
-      </c>
-      <c r="H14" s="20" t="inlineStr">
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Vivienne_Pham/Week_of_2026-02-16/ ✓ ✓</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
         <is>
           <t>2026-02-22</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="11">
-      <c r="C15" s="10" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Vivienne Pham</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>24</v>
+      </c>
+      <c r="E17" t="n">
+        <v>88</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>3 boards | 9 roles (3 archetypes) | NYC, DC, Remote</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Vivienne_Pham/Week_of_2026-02-23/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>2026-02-22</t>
         </is>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D18" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E18" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>4 boards | 9 roles (3 archetypes) | NYC, DC, Remote</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>Vivienne_Pham/Week_of_2026-02-16/</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="11">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Rosalind Gahamire</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>2026-02-18</t>
         </is>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D19" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E19" s="10" t="n">
         <v>87</v>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Greenhouse/Lever/Ashby/LinkedIn | Brand Strategist, Creative Strategist, Marketing Manager | Lisbon, Remote-Global/EMEA</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
         <is>
           <t>2026-02-23 ✓</t>
         </is>
       </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Rosalind_Gahamire/Week_of_2026-02-16/</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="C17" s="10" t="inlineStr">
+    <row r="20">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>2026-02-22</t>
         </is>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D20" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E20" s="10" t="n">
         <v>87</v>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>4 boards | Brand/Creative Strategy, Marketing Mgr | Lisbon, Remote-Global</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>Rosalind_Gahamire/Week_of_2026-02-16/</t>
         </is>

</xml_diff>